<commit_message>
update: SF_2 result (Spain 2-1 Belgium) + H2H data + teams.json ranking update
- knockout_bracket: add SF_2, fix teamB Germany->Belgium
- historical.csv: add France-Spain H2H (3 matches), fix GBK->UTF-8 encoding
- teams.json: Spain fifaRank 3->2, Argentina fifaRank 2->3
- looking_ahead.xlsx: 11 match analysis blocks (incl. remaining SFs)
- Regenerated predictions: France 52.7%, Norway 15.7%, Spain 14.0%
</commit_message>
<xml_diff>
--- a/backend/data/looking_ahead.xlsx
+++ b/backend/data/looking_ahead.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="188">
   <si>
     <t>国家</t>
   </si>
@@ -557,6 +557,42 @@
   </si>
   <si>
     <t>世界杯曾0-1负阿根廷，处于下风</t>
+  </si>
+  <si>
+    <t>稳居世界顶级强队，夺冠热门之一</t>
+  </si>
+  <si>
+    <t>欧洲中游球队，队史首进世界杯八强</t>
+  </si>
+  <si>
+    <t>总身价13.6亿欧元，阵容厚度碾压对手</t>
+  </si>
+  <si>
+    <t>总身价5.9亿欧元，依赖哈兰德、厄德高</t>
+  </si>
+  <si>
+    <t>连克强敌，凯恩6球，贝林厄姆状态火热</t>
+  </si>
+  <si>
+    <t>淘汰巴西士气高涨，哈兰德4场7球</t>
+  </si>
+  <si>
+    <t>宽萨红牌停赛，格伊、赖斯和詹姆斯参加最后一轮合练</t>
+  </si>
+  <si>
+    <t>否认流感传闻，26名球员全员参加训练</t>
+  </si>
+  <si>
+    <t>控球主导，边路突破中路渗透结合</t>
+  </si>
+  <si>
+    <t>541防守反击，边路传中找哈兰德</t>
+  </si>
+  <si>
+    <t>图赫尔战术灵活，大赛经验丰富</t>
+  </si>
+  <si>
+    <t>索尔巴肯务实，善用反击和定位球</t>
   </si>
 </sst>
 </file>
@@ -1490,11 +1526,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9.24778761061947" style="1" customWidth="1"/>
-    <col min="2" max="2" width="40.787610619469" style="1" customWidth="1"/>
+    <col min="2" max="2" width="52.2743362831858" style="1" customWidth="1"/>
     <col min="3" max="3" width="43.6283185840708" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2420,6 +2456,83 @@
       </c>
       <c r="C93" s="1" t="s">
         <v>175</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: SF_3/SF_4 results (England, Argentina advance) + final previews
- knockout_bracket: SF_3 挪威1:2英格兰, SF_4 阿根廷3:1瑞士
- looking_ahead.xlsx: 13 match analyses (added F_1 法国vs西班牙, F_2 英格兰vs阿根廷)
- Regenerated predictions: France 57.1%, Spain 15.4%, England 14.5%, Argentina 13.0%
- 4 teams remaining, model accuracy 74/100
</commit_message>
<xml_diff>
--- a/backend/data/looking_ahead.xlsx
+++ b/backend/data/looking_ahead.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="221">
   <si>
     <t>国家</t>
   </si>
@@ -593,6 +593,105 @@
   </si>
   <si>
     <t>索尔巴肯务实，善用反击和定位球</t>
+  </si>
+  <si>
+    <t>总身价15.2亿欧元，本届赛事最高</t>
+  </si>
+  <si>
+    <t>总身价12.2亿欧元，阵容价值高昂</t>
+  </si>
+  <si>
+    <t>6战全胜轰16球，进攻效率顶尖</t>
+  </si>
+  <si>
+    <t>6战仅失1球，曾创650分钟零封纪录</t>
+  </si>
+  <si>
+    <t>姆巴佩8球3助攻，脚踝轻伤影响有限</t>
+  </si>
+  <si>
+    <t>尼科伤缺边路受损，其余主力健康</t>
+  </si>
+  <si>
+    <t>战术打法</t>
+  </si>
+  <si>
+    <t>防守反击犀利，依赖个人速度爆破</t>
+  </si>
+  <si>
+    <t>极致传控，中场控制力极强</t>
+  </si>
+  <si>
+    <t>近期交锋</t>
+  </si>
+  <si>
+    <t>2021欧国联决赛曾击败西班牙</t>
+  </si>
+  <si>
+    <t>近两次大赛半决赛均淘汰法国</t>
+  </si>
+  <si>
+    <t>阵容深度</t>
+  </si>
+  <si>
+    <t>三线均有世界级替补，轮换选择多</t>
+  </si>
+  <si>
+    <t>边路伤病后轮换深度不足</t>
+  </si>
+  <si>
+    <t>教练风格</t>
+  </si>
+  <si>
+    <t>德尚务实稳重，大赛抗压能力强</t>
+  </si>
+  <si>
+    <t>德拉富恩特主打传控，战术激进</t>
+  </si>
+  <si>
+    <t>实力强劲，阵容均衡，攻防两端无明显短板</t>
+  </si>
+  <si>
+    <t>实力稳居前三，卫冕冠军，大赛韧性极强</t>
+  </si>
+  <si>
+    <t>总身价13.2亿欧元，阵容豪华</t>
+  </si>
+  <si>
+    <t>总身价7.8亿欧元，核心球员价值突出</t>
+  </si>
+  <si>
+    <t>小组头名出线，淘汰赛连克强敌，贝林厄姆6球</t>
+  </si>
+  <si>
+    <t>小组赛全胜，淘汰赛多次逆转，梅西8球领跑</t>
+  </si>
+  <si>
+    <t>凯恩巅峰稳定，贝林厄姆攻防一体，状态火热</t>
+  </si>
+  <si>
+    <t>梅西核心作用无可替代，马丁内斯扑点顶级</t>
+  </si>
+  <si>
+    <t>赖斯、格希等有轻微伤情，整体影响有限</t>
+  </si>
+  <si>
+    <t>梅西、恩佐等核心疲劳，无严重伤病</t>
+  </si>
+  <si>
+    <t>平均年龄更低，轮换充足，体能储备占优</t>
+  </si>
+  <si>
+    <t>后防老龄化，替补深度不足，后半程体能堪忧</t>
+  </si>
+  <si>
+    <t>4231高位逼抢，边路冲击+中路渗透结合</t>
+  </si>
+  <si>
+    <t>442控球反击，依托梅西组织，转换高效</t>
+  </si>
+  <si>
+    <t>斯卡洛尼务实稳重，大赛执教经验丰富</t>
   </si>
 </sst>
 </file>
@@ -1526,7 +1625,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9.24778761061947" style="1" customWidth="1"/>
@@ -2533,6 +2632,190 @@
       </c>
       <c r="C101" s="1" t="s">
         <v>187</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3">
+      <c r="A103" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3">
+      <c r="A104" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3">
+      <c r="A106" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3">
+      <c r="A107" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3">
+      <c r="A118" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3">
+      <c r="A120" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
@ data: 更新前瞻数据 looking_ahead.xlsx（14场前瞻）
Co-Authored-By: Claude <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/backend/data/looking_ahead.xlsx
+++ b/backend/data/looking_ahead.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="240">
   <si>
     <t>国家</t>
   </si>
@@ -691,7 +691,64 @@
     <t>442控球反击，依托梅西组织，转换高效</t>
   </si>
   <si>
+    <t>图赫尔战术灵活，擅长临场调整与控场</t>
+  </si>
+  <si>
     <t>斯卡洛尼务实稳重，大赛执教经验丰富</t>
+  </si>
+  <si>
+    <t>稳居世界前三，攻防均衡无明显短板</t>
+  </si>
+  <si>
+    <t>稳居世界前十，传控体系成熟稳定</t>
+  </si>
+  <si>
+    <t>总身价15.2亿欧元，足坛第一</t>
+  </si>
+  <si>
+    <t>总身价13.1亿欧元，足坛第二</t>
+  </si>
+  <si>
+    <t>6战全胜进16球失2球，淘汰赛三连零封</t>
+  </si>
+  <si>
+    <t>5胜1平进11球失1球，防线稳固</t>
+  </si>
+  <si>
+    <t>姆巴佩8球3助，登贝莱5球，状态火热</t>
+  </si>
+  <si>
+    <t>亚马尔2球3助，奥亚萨瓦尔4球，罗德里控场</t>
+  </si>
+  <si>
+    <t>姆巴佩轻微脚踝挫伤，楚阿梅尼伤愈</t>
+  </si>
+  <si>
+    <t>尼科·威廉姆斯伤缺，其余主力健康</t>
+  </si>
+  <si>
+    <t>板凳深度断层领先，两套首发无缝轮换</t>
+  </si>
+  <si>
+    <t>轮换充足，但锋线终结能力存疑</t>
+  </si>
+  <si>
+    <t>务实反击高效，抓防线身后空档</t>
+  </si>
+  <si>
+    <t>高位传控压迫，控球率高达65%</t>
+  </si>
+  <si>
+    <t>德尚务实强硬，大赛经验丰富</t>
+  </si>
+  <si>
+    <t>德拉富恩特善用年轻球员，传控大师</t>
+  </si>
+  <si>
+    <t>近两次半决赛负于西班牙，需复仇</t>
+  </si>
+  <si>
+    <t>近两次半决赛击败法国，心理占优</t>
   </si>
 </sst>
 </file>
@@ -1625,7 +1682,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9.24778761061947" style="1" customWidth="1"/>
@@ -2814,8 +2871,121 @@
       <c r="A120" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="B120" s="1" t="s">
+        <v>220</v>
+      </c>
       <c r="C120" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3">
+      <c r="A124" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3">
+      <c r="A126" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3">
+      <c r="A127" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3">
+      <c r="A128" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3">
+      <c r="A129" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3">
+      <c r="A130" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
@ fix: historical.csv编码自动检测(UTF-8/GBK) + 数据更新
- features.py / model.py: 读取historical.csv自动尝试UTF-8和GBK编码
- 更新前瞻数据 + 历史数据

Co-Authored-By: Claude <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/backend/data/looking_ahead.xlsx
+++ b/backend/data/looking_ahead.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20152" windowHeight="10125"/>
+    <workbookView windowWidth="22192" windowHeight="10717"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="287">
   <si>
     <t>国家</t>
   </si>
@@ -806,6 +806,90 @@
   </si>
   <si>
     <t>半决赛5战全胜，对英淘汰赛2战全胜</t>
+  </si>
+  <si>
+    <t>总身价15.2亿欧元，锋线豪华全球居首</t>
+  </si>
+  <si>
+    <t>总身价13.2亿欧元，年轻球星云集</t>
+  </si>
+  <si>
+    <t>6胜1负进16球，半决赛不敌西班牙</t>
+  </si>
+  <si>
+    <t>4胜2平1负进13球，半决赛遭阿根廷绝杀</t>
+  </si>
+  <si>
+    <t>姆巴佩8球领跑射手榜，带伤作战</t>
+  </si>
+  <si>
+    <t>凯恩、贝林厄姆各6球，核心稳定</t>
+  </si>
+  <si>
+    <t>姆巴佩脚踝有伤，无其他核心伤缺</t>
+  </si>
+  <si>
+    <t>宽萨停赛，里斯·詹姆斯存疑</t>
+  </si>
+  <si>
+    <t>淘汰赛轮换充分，体能储备更佳</t>
+  </si>
+  <si>
+    <t>多场加时鏖战，主力消耗严重</t>
+  </si>
+  <si>
+    <t>收缩反击犀利，边路突破威胁大</t>
+  </si>
+  <si>
+    <t>阵地进攻为主，边路传中找凯恩</t>
+  </si>
+  <si>
+    <t>德尚防守反击体系成熟，大赛经验足</t>
+  </si>
+  <si>
+    <t>图赫尔战术灵活，临场调整强</t>
+  </si>
+  <si>
+    <t>7战6胜1平仅失1球，零封5场，状态火热</t>
+  </si>
+  <si>
+    <t>7战全胜，多次逆转，韧性极强</t>
+  </si>
+  <si>
+    <t>亚马尔边路犀利，罗德里中场攻防核心</t>
+  </si>
+  <si>
+    <t>梅西8球4助攻，大赛关键先生</t>
+  </si>
+  <si>
+    <t>伤病体能</t>
+  </si>
+  <si>
+    <t>无伤病，平均年龄26.3岁，体能充沛</t>
+  </si>
+  <si>
+    <t>无伤病，主力高龄，多场加时体能堪忧</t>
+  </si>
+  <si>
+    <t>阵容身价</t>
+  </si>
+  <si>
+    <t>总身价约12.2亿欧元，阵容深度厚</t>
+  </si>
+  <si>
+    <t>总身价约7.8亿欧元，核心班底稳定</t>
+  </si>
+  <si>
+    <t>改良传控，高位压迫，中场控制力强</t>
+  </si>
+  <si>
+    <t>低位防守，快速反击，专克传控</t>
+  </si>
+  <si>
+    <t>德拉富恩特务实，攻守转换效率高</t>
+  </si>
+  <si>
+    <t>斯卡洛尼擅长逆风球，战术针对性强</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1823,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C159"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9.24778761061947" style="1" customWidth="1"/>
@@ -3153,6 +3237,171 @@
       </c>
       <c r="C142" s="1" t="s">
         <v>258</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3">
+      <c r="A144" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3">
+      <c r="A145" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3">
+      <c r="A146" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3">
+      <c r="A147" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3">
+      <c r="A148" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3">
+      <c r="A150" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3">
+      <c r="A151" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3">
+      <c r="A153" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3">
+      <c r="A154" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3">
+      <c r="A155" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3">
+      <c r="A156" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3">
+      <c r="A157" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3">
+      <c r="A158" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3">
+      <c r="A159" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>